<commit_message>
Remove sample student data and privacy defaults
</commit_message>
<xml_diff>
--- a/docs/student-import-template.xlsx
+++ b/docs/student-import-template.xlsx
@@ -128,120 +128,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr" s="0">
-        <is>
-          <t>冯成妍</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr" s="0">
-        <is>
-          <t>IELTS</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr" s="0">
-        <is>
-          <t>中等</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr" s="0">
-        <is>
-          <t>IELTS 5.5</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr" s="0">
-        <is>
-          <t>6.5</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr" s="0">
-        <is>
-          <t>2026-06-15</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr" s="0">
-        <is>
-          <t>雅思1v1</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr" s="0">
-        <is>
-          <t>雅思1v1-30课时</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr" s="0">
-        <is>
-          <t>30</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr" s="0">
-        <is>
-          <t>Polla</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr" s="0">
-        <is>
-          <t>示例：6月考试，注意阅读重复刷题</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr" s="0">
-        <is>
-          <t>刘珈绮</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr" s="0">
-        <is>
-          <t>IELTS</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr" s="0">
-        <is>
-          <t>较稳</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr" s="0">
-        <is>
-          <t>IELTS 6.0</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr" s="0">
-        <is>
-          <t>7.0</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr" s="0">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr" s="0">
-        <is>
-          <t>雅思班课</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr" s="0">
-        <is>
-          <t>雅思脱产班（秋季）</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr" s="0">
-        <is>
-          <t>80</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr" s="0">
-        <is>
-          <t>其他助教</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr" s="0">
-        <is>
-          <t>示例：班课学生，统一按班课标签显示</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -390,7 +276,7 @@
       </c>
       <c r="B11" t="inlineStr" s="0">
         <is>
-          <t>默认 Polla，也可以填其他助教姓名。</t>
+          <t>可填助教A、其他助教，或留空显示未匹配。</t>
         </is>
       </c>
     </row>

</xml_diff>